<commit_message>
feat(form): add Email question to Daily Activity Report (submitter notifications)
</commit_message>
<xml_diff>
--- a/koboforms/KF-Daily_Activity_Report.xlsx
+++ b/koboforms/KF-Daily_Activity_Report.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -610,36 +610,40 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>email</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>District</t>
+          <t>Your email (to receive approval / rejection notice)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>We email you if a manager approves or rejects this entry.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>any_activity</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Did you have any patients / activity today?</t>
+          <t>District</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -653,50 +657,74 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>activity_note</t>
+          <t>any_activity</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Brief note on today’s activity</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>${any_activity}='yes'</t>
-        </is>
-      </c>
+          <t>Did you have any patients / activity today?</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>zero_note</t>
+          <t>activity_note</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>You are submitting a ZERO report — no activity recorded today. This still counts as your daily report.</t>
+          <t>Brief note on today’s activity</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
+          <t>${any_activity}='yes'</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>zero_note</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>You are submitting a ZERO report — no activity recorded today. This still counts as your daily report.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>${any_activity}='no'</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>